<commit_message>
Untrack Excel lock file, ignore ~$* temp files, update dependency sheet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mv_dependency_sheet.xlsx
+++ b/mv_dependency_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Warehouse Work\CHT\community_health_datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7D3DF2-D789-4ACC-9D3B-CAD2021B4626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67C7D23E-9F10-4D62-8102-A02A68A9C10F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{7B169CB4-C442-4F28-981F-E3FEB42AE81D}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
   <si>
     <t>MV</t>
   </si>
@@ -69,6 +69,18 @@
   </si>
   <si>
     <t>cht.mv_cebs_signal_verification</t>
+  </si>
+  <si>
+    <t>cht.mv_delivery_report</t>
+  </si>
+  <si>
+    <t>cht.mv_delivery</t>
+  </si>
+  <si>
+    <t>cht.mv_pregnancy</t>
+  </si>
+  <si>
+    <t>check</t>
   </si>
 </sst>
 </file>
@@ -506,15 +518,36 @@
       <c r="C4" t="s">
         <v>3</v>
       </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">

</xml_diff>